<commit_message>
Ajoute fiches, observations et frise de médicaments au dossier patient
- Deux nouveaux onglets dans Documents (Fiches, Observations médicales),
  affichage en accordéon (titre/date/UF), utilisables comme source de
  suggestions de codage avec surlignage automatique à la navigation.
- Onglet Médicaments reconstruit en grille jour par jour scrollable
  (administrations réelles) avec tableau de détail, alimentée par une
  nouvelle table administrations.xlsx générée depuis la fréquence de
  chaque médicament.
- Panneau de codage rétractable et à défilement indépendant : la barre
  supérieure reste toujours visible.
- L'onglet actif et le défilement de la barre des séjours sont conservés
  au changement de séjour/patient.
- README mis à jour (démarrage rapide, nouvelles tables Excel, résumé des
  évolutions UI).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/documents.xlsx
+++ b/data/documents.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,15 +466,20 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>uf</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>excerpt</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>full_text</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>highlight</t>
         </is>
@@ -518,15 +523,20 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>UF Cardiologie</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>Patiente admise pour décompensation cardiaque globale sur cardiopathie ischémique connue, avec insuffisance rénale aiguë sur chronique stade IIIB. Évolution favorable sous traitement diurétique IV.</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Patiente admise pour décompensation cardiaque globale sur cardiopathie ischémique connue, avec insuffisance rénale aiguë sur chronique stade IIIB. Évolution favorable sous traitement diurétique IV. Le bilan biologique d'entrée retrouvait un NT-proBNP à 5400 ng/L et une créatininémie à 142 µmol/L. L'échocardiographie a confirmé une dysfonction ventriculaire gauche sévère (FEVG 30%). Traitement diurétique intraveineux avec surveillance stricte de la diurèse, permettant une amélioration clinique et biologique progressive. Sortie à domicile avec majoration du traitement de fond et mise en place d'une hospitalisation à domicile (HAD).</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>cardiopathie ischémique</t>
         </is>
@@ -570,15 +580,20 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>UF Imagerie cardiaque</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>FEVG estimée à 30%, hypokinésie globale. Pas d'épanchement péricardique. Valves sans anomalie significative.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>FEVG estimée à 30%, hypokinésie globale. Pas d'épanchement péricardique. Valves sans anomalie significative. Cinétique globale altérée de façon homogène, sans anomalie segmentaire focale évocatrice d'une séquelle territoriale univoque. Fonction diastolique non évaluable de façon fiable dans ce contexte.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>FEVG estimée à 30%</t>
         </is>
@@ -622,15 +637,20 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>UF Cardiologie</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>Poids stable à 68kg, auscultation pulmonaire libre. Poursuite du traitement, kaliémie basse à surveiller.</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Poids stable à 68kg, auscultation pulmonaire libre. Poursuite du traitement, kaliémie basse à surveiller. Le traitement bêta-bloquant et l'IEC ont été maintenus à dose stable. Surveillance rapprochée du ionogramme prévue en ville dans les 15 jours compte tenu de la kaliémie basse.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>kaliémie basse</t>
         </is>
@@ -674,15 +694,20 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>UF Cardiologie interventionnelle</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>Sténose serrée de l'artère interventriculaire antérieure proximale, traitée par angioplastie et pose d'un stent actif.</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Sténose serrée de l'artère interventriculaire antérieure proximale, traitée par angioplastie et pose d'un stent actif. Angioplastie réalisée avec succès par voie radiale droite, sans complication au point de ponction. Double antiagrégation plaquettaire instaurée pour une durée de 12 mois.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>stent actif</t>
         </is>
@@ -726,15 +751,20 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
+          <t>UF Pneumologie</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>Pneumopathie basale droite d'allure bactérienne, syndrome inflammatoire biologique marqué à l'entrée. Évolution favorable sous antibiothérapie.</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Pneumopathie basale droite d'allure bactérienne, syndrome inflammatoire biologique marqué à l'entrée. Évolution favorable sous antibiothérapie. Hémocultures négatives, antigénurie légionelle et pneumocoque négatives. Antibiothérapie probabiliste par amoxicilline-acide clavulanique avec relais oral à J5, bonne évolution clinique et biologique.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Pneumopathie basale droite</t>
         </is>
@@ -778,15 +808,20 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
+          <t>UF Imagerie</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
           <t>Foyer de condensation alvéolaire du lobe inférieur droit, sans épanchement pleural associé.</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Foyer de condensation alvéolaire du lobe inférieur droit, sans épanchement pleural associé. Contrôle radiologique de sortie non réalisé, à prévoir à distance si persistance de symptômes.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>foyer de condensation alvéolaire</t>
         </is>
@@ -830,15 +865,20 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
+          <t>UF Pneumologie</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
           <t>Pneumopathie basale gauche, évolution favorable sous antibiothérapie orale.</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Pneumopathie basale gauche, évolution favorable sous antibiothérapie orale. Évolution rapidement favorable sous antibiothérapie orale d'emblée, sans nécessité d'oxygénothérapie.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Pneumopathie basale gauche</t>
         </is>
@@ -882,15 +922,20 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
+          <t>UF Bloc opératoire</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
           <t>Mise en place d'une prothèse totale de hanche non cimentée, voie postéro-externe, sans incident peropératoire. Pertes sanguines estimées à 250mL.</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Mise en place d'une prothèse totale de hanche non cimentée, voie postéro-externe, sans incident peropératoire. Pertes sanguines estimées à 250mL. Intervention réalisée sous rachianesthésie, durée opératoire de 55 minutes. Aucune transfusion peropératoire nécessaire. Suites immédiates simples.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>prothèse totale de hanche</t>
         </is>
@@ -934,15 +979,20 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
+          <t>UF Chirurgie orthopédique</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
           <t>Patient sortant avec appui partiel, traitement antalgique et anticoagulant préventif pendant 35 jours.</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Patient sortant avec appui partiel, traitement antalgique et anticoagulant préventif pendant 35 jours. Consignes de rééducation transmises au centre de SSR, avec limitation de la flexion de hanche au-delà de 90° pendant 6 semaines.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>anticoagulant préventif</t>
         </is>
@@ -986,15 +1036,20 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
+          <t>UF Chirurgie orthopédique</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
           <t>Coxarthrose évoluée symptomatique, indication de prothèse totale de hanche retenue.</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Coxarthrose évoluée symptomatique, indication de prothèse totale de hanche retenue. Bilan pré-anesthésique programmé, absence de contre-indication à l'intervention à ce stade.</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>prothèse totale de hanche</t>
         </is>

</xml_diff>